<commit_message>
re do of roundup bc it was not saved
</commit_message>
<xml_diff>
--- a/week-01/Ex2B_roundup.xlsx
+++ b/week-01/Ex2B_roundup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thaniastaana\DataAnalytics\week-01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{153AD06E-A785-4371-929F-3CC82E8F02D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F4C01D0F-F173-4A92-A869-4E1D4060459B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="1560" windowWidth="15252" windowHeight="7884" xr2:uid="{8C2B0283-67EE-4770-AF27-B7C074AF6CAB}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8C2B0283-67EE-4770-AF27-B7C074AF6CAB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,6 +36,50 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="13">
+  <si>
+    <t>LinkedIn</t>
+  </si>
+  <si>
+    <t>Social Media</t>
+  </si>
+  <si>
+    <t>Can choose what you want to download</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>go to "me" icon and select "settings and privacy" and click "data privacy". Under "how linkedin uses your data section", click "download your data" choose which specific data or all and then click "request archive"</t>
+  </si>
+  <si>
+    <t>CSV</t>
+  </si>
+  <si>
+    <t>Reddit</t>
+  </si>
+  <si>
+    <t>Posts, comments, saved posts and comments, chat history and messages</t>
+  </si>
+  <si>
+    <t>go to official data request page and log into account. Choose request settings and submit the request. Wait for reddit to process file and then they will DM you the download link</t>
+  </si>
+  <si>
+    <t>Instagram</t>
+  </si>
+  <si>
+    <t>can choose how much and how little you want to cover. Can edit what you want and the time duration</t>
+  </si>
+  <si>
+    <t>JSON or HTML</t>
+  </si>
+  <si>
+    <t>go to account center and click "your information and permissions" and select "export your information" and then "create export" and to export to device or other</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -69,8 +113,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -405,9 +455,77 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF297F7E-AE47-4CBF-8B04-3F8EDB5F38C4}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="15.6640625" customWidth="1"/>
+    <col min="3" max="3" width="25.109375" customWidth="1"/>
+    <col min="5" max="5" width="35.77734375" customWidth="1"/>
+    <col min="6" max="6" width="13.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="144" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" s="1"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>